<commit_message>
Minor update: extra row for mining hardware compatibility, also changed screenshot
</commit_message>
<xml_diff>
--- a/2minuteblock_vs_infrablock_vs_tailstorm_comparison.xlsx
+++ b/2minuteblock_vs_infrablock_vs_tailstorm_comparison.xlsx
@@ -13,14 +13,14 @@
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1"/>
+      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="126">
   <si>
     <t xml:space="preserve">2-minute Blocks</t>
   </si>
@@ -396,6 +396,12 @@
   </si>
   <si>
     <t xml:space="preserve">Will wallets need to be modified so that the upgrade can work?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mining with Existing Hardware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is ASIC mining possible without changes?</t>
   </si>
   <si>
     <t xml:space="preserve">Miner Revenue</t>
@@ -1517,34 +1523,37 @@
       <c r="B12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>44</v>
+      <c r="C12" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>22</v>
       </c>
+      <c r="H12" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D13" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>47</v>
+      <c r="E13" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>16</v>
@@ -1552,22 +1561,19 @@
       <c r="G13" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>48</v>
-      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>51</v>
+      <c r="D14" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>16</v>
@@ -1576,56 +1582,56 @@
         <v>22</v>
       </c>
       <c r="H14" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="14" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="14"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="14"/>
-      <c r="G15" s="7"/>
+      <c r="D15" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G16" s="9"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="14"/>
+      <c r="G16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E17" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="H17" s="2" t="s">
+      <c r="C18" s="6" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="2" t="s">
+      <c r="D18" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>22</v>
+      <c r="E18" s="6" t="s">
+        <v>57</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>16</v>
@@ -1634,21 +1640,21 @@
         <v>22</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>22</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>63</v>
+        <v>61</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>16</v>
@@ -1657,21 +1663,21 @@
         <v>22</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>22</v>
+      <c r="D20" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>65</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>16</v>
@@ -1683,15 +1689,15 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="14" t="s">
-        <v>68</v>
+      <c r="D21" s="9" t="s">
+        <v>22</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>22</v>
@@ -1703,22 +1709,37 @@
         <v>22</v>
       </c>
       <c r="H21" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G22" s="9"/>
+      <c r="C22" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G23" s="9"/>
     </row>
-    <row r="25" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>71</v>
-      </c>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G24" s="9"/>
     </row>
     <row r="26" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
@@ -1744,93 +1765,81 @@
         <v>77</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="16"/>
-    </row>
-    <row r="30" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="16" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="16"/>
+      <c r="L30" s="16"/>
+      <c r="M30" s="16"/>
+      <c r="N30" s="16"/>
+    </row>
+    <row r="31" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="17"/>
-      <c r="L32" s="17"/>
-      <c r="M32" s="17"/>
-      <c r="N32" s="17"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
+      <c r="L32" s="16"/>
+      <c r="M32" s="16"/>
+      <c r="N32" s="16"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="16"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="17"/>
+      <c r="K33" s="17"/>
+      <c r="L33" s="17"/>
+      <c r="M33" s="17"/>
+      <c r="N33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
@@ -1852,13 +1861,25 @@
       <c r="M34" s="16"/>
       <c r="N34" s="16"/>
     </row>
-    <row r="35" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="16" t="s">
         <v>91</v>
       </c>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16"/>
     </row>
     <row r="36" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
@@ -1884,53 +1905,41 @@
         <v>97</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="B39" s="16" t="s">
+      <c r="B39" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="16"/>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="16"/>
-    </row>
-    <row r="40" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="16" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
+      <c r="L40" s="16"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="16"/>
+    </row>
+    <row r="41" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="B41" s="16" t="s">
+      <c r="B41" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C41" s="16"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-      <c r="F41" s="16"/>
-      <c r="G41" s="16"/>
-      <c r="H41" s="16"/>
-      <c r="I41" s="16"/>
-      <c r="J41" s="16"/>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="15" t="s">
@@ -2033,48 +2042,54 @@
       <c r="N46" s="16"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15"/>
-      <c r="B47" s="16"/>
+      <c r="A47" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="B47" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="16"/>
+      <c r="L47" s="16"/>
+      <c r="M47" s="16"/>
+      <c r="N47" s="16"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="18" t="s">
-        <v>114</v>
-      </c>
+      <c r="A48" s="15"/>
+      <c r="B48" s="16"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="16"/>
+      <c r="B49" s="18" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="15"/>
-      <c r="F50" s="15"/>
-      <c r="G50" s="15"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="20"/>
-      <c r="J50" s="20"/>
-      <c r="K50" s="20"/>
+      <c r="B50" s="16"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="C51" s="21"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="21"/>
-      <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
-      <c r="H51" s="21"/>
-      <c r="I51" s="21"/>
-      <c r="J51" s="21"/>
-      <c r="K51" s="21"/>
+      <c r="B51" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+      <c r="H51" s="20"/>
+      <c r="I51" s="20"/>
+      <c r="J51" s="20"/>
+      <c r="K51" s="20"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C52" s="21"/>
       <c r="D52" s="21"/>
@@ -2084,38 +2099,38 @@
       <c r="H52" s="21"/>
       <c r="I52" s="21"/>
       <c r="J52" s="21"/>
-      <c r="K52" s="20"/>
+      <c r="K52" s="21"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="20" t="s">
-        <v>118</v>
-      </c>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="20"/>
-      <c r="F53" s="20"/>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="20"/>
-      <c r="J53" s="20"/>
+      <c r="B53" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="C53" s="21"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="21"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="21"/>
+      <c r="H53" s="21"/>
+      <c r="I53" s="21"/>
+      <c r="J53" s="21"/>
       <c r="K53" s="20"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="20"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
+      <c r="B54" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C54" s="20"/>
+      <c r="D54" s="20"/>
+      <c r="E54" s="20"/>
+      <c r="F54" s="20"/>
+      <c r="G54" s="20"/>
       <c r="H54" s="20"/>
       <c r="I54" s="20"/>
       <c r="J54" s="20"/>
       <c r="K54" s="20"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="22" t="s">
-        <v>119</v>
-      </c>
+      <c r="B55" s="20"/>
       <c r="C55" s="15"/>
       <c r="D55" s="15"/>
       <c r="E55" s="15"/>
@@ -2127,74 +2142,87 @@
       <c r="K55" s="20"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
-      <c r="E56" s="20"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="20"/>
+      <c r="B56" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
       <c r="H56" s="20"/>
       <c r="I56" s="20"/>
       <c r="J56" s="20"/>
       <c r="K56" s="20"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="C57" s="23"/>
-      <c r="D57" s="23"/>
-      <c r="E57" s="23"/>
-      <c r="F57" s="23"/>
-      <c r="G57" s="23"/>
-      <c r="H57" s="23"/>
-      <c r="I57" s="23"/>
-      <c r="J57" s="23"/>
-      <c r="K57" s="23"/>
+      <c r="B57" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="C57" s="20"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="20"/>
+      <c r="F57" s="20"/>
+      <c r="G57" s="20"/>
+      <c r="H57" s="20"/>
+      <c r="I57" s="20"/>
+      <c r="J57" s="20"/>
+      <c r="K57" s="20"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="20"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="15"/>
-      <c r="F58" s="15"/>
-      <c r="G58" s="15"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="20"/>
-      <c r="J58" s="20"/>
-      <c r="K58" s="20"/>
+      <c r="B58" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="C58" s="23"/>
+      <c r="D58" s="23"/>
+      <c r="E58" s="23"/>
+      <c r="F58" s="23"/>
+      <c r="G58" s="23"/>
+      <c r="H58" s="23"/>
+      <c r="I58" s="23"/>
+      <c r="J58" s="23"/>
+      <c r="K58" s="23"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="C59" s="22"/>
-      <c r="D59" s="22"/>
-      <c r="E59" s="22"/>
-      <c r="F59" s="22"/>
-      <c r="G59" s="22"/>
-      <c r="H59" s="22"/>
-      <c r="I59" s="22"/>
-      <c r="J59" s="22"/>
-      <c r="K59" s="22"/>
+      <c r="B59" s="20"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="20"/>
+      <c r="I59" s="20"/>
+      <c r="J59" s="20"/>
+      <c r="K59" s="20"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
-      <c r="E60" s="20"/>
-      <c r="F60" s="20"/>
-      <c r="G60" s="20"/>
-      <c r="H60" s="20"/>
-      <c r="I60" s="20"/>
-      <c r="J60" s="20"/>
-      <c r="K60" s="20"/>
-    </row>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="B60" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="C60" s="22"/>
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="22"/>
+      <c r="H60" s="22"/>
+      <c r="I60" s="22"/>
+      <c r="J60" s="22"/>
+      <c r="K60" s="22"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="C61" s="20"/>
+      <c r="D61" s="20"/>
+      <c r="E61" s="20"/>
+      <c r="F61" s="20"/>
+      <c r="G61" s="20"/>
+      <c r="H61" s="20"/>
+      <c r="I61" s="20"/>
+      <c r="J61" s="20"/>
+      <c r="K61" s="20"/>
+    </row>
     <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2203,7 +2231,6 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="B25:N25"/>
     <mergeCell ref="B26:N26"/>
     <mergeCell ref="B27:N27"/>
     <mergeCell ref="B28:N28"/>
@@ -2225,23 +2252,24 @@
     <mergeCell ref="B44:N44"/>
     <mergeCell ref="B45:N45"/>
     <mergeCell ref="B46:N46"/>
-    <mergeCell ref="B51:K51"/>
-    <mergeCell ref="B52:J52"/>
+    <mergeCell ref="B47:N47"/>
+    <mergeCell ref="B52:K52"/>
     <mergeCell ref="B53:J53"/>
-    <mergeCell ref="B56:K56"/>
+    <mergeCell ref="B54:J54"/>
     <mergeCell ref="B57:K57"/>
-    <mergeCell ref="B59:K59"/>
+    <mergeCell ref="B58:K58"/>
     <mergeCell ref="B60:K60"/>
+    <mergeCell ref="B61:K61"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B57" r:id="rId1" display="https://gitlab.com/ShadowOfHarbringer/infrastructureblocks/-/raw/master/implementation_consequences_v1.5.pdf?ref_type=heads&amp;inline=false"/>
+    <hyperlink ref="B58" r:id="rId1" display="https://gitlab.com/ShadowOfHarbringer/infrastructureblocks/-/raw/master/implementation_consequences_v1.5.pdf?ref_type=heads&amp;inline=false"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normalny"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normalny"&amp;12Strona &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CStrona &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update 2025-20-03: Added stakeholder effort to implement + minor bugfixes
</commit_message>
<xml_diff>
--- a/2minuteblock_vs_infrablock_vs_tailstorm_comparison.xlsx
+++ b/2minuteblock_vs_infrablock_vs_tailstorm_comparison.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="156">
   <si>
     <t xml:space="preserve">2-minute Blocks</t>
   </si>
@@ -372,6 +372,9 @@
     <t xml:space="preserve">Wallet Compatibility Affected</t>
   </si>
   <si>
+    <t xml:space="preserve">Minimally</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -401,7 +404,7 @@
     <t xml:space="preserve">Mining with Existing Hardware</t>
   </si>
   <si>
-    <t xml:space="preserve">Is ASIC mining possible without changes?</t>
+    <t xml:space="preserve">Is ASIC mining possible?</t>
   </si>
   <si>
     <t xml:space="preserve">Miner Revenue</t>
@@ -410,7 +413,24 @@
     <t xml:space="preserve">Small decrease</t>
   </si>
   <si>
-    <t xml:space="preserve">Increase</t>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF00A933"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Increase </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF00A933"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(23)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Solo Mining Profitability</t>
@@ -636,6 +656,137 @@
     <t xml:space="preserve">How will market &amp; speculation activity on CEXes &amp; DEXes be affected by a proposal</t>
   </si>
   <si>
+    <t xml:space="preserve">Stakeholder’s Effort to Implement:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Very Rough Estimation) Which stakeholders will have to do how much work after the proposal is implemented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node Software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scale: None &lt; Very Low &lt; Low &lt; Medium &lt; High &lt; Very High &lt; Massive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol Libraries and Tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wallets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very Low to Low</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF2A6099"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">None → Low/Medium </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF2A6099"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(24)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium to High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centralized Exchanges</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF2A6099"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">None → Medium </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF2A6099"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(24)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEXes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment Operators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASIC Miners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None to Very Low </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF158466"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Low to Medium </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF158466"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(25)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Unpredictable </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(26)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Block Explorers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High to Very High</t>
+  </si>
+  <si>
     <t xml:space="preserve">(1)</t>
   </si>
   <si>
@@ -681,7 +832,7 @@
     <t xml:space="preserve">(8)</t>
   </si>
   <si>
-    <t xml:space="preserve">Orphan rate and all other basic properties of main chain remain unchanged, any significant changes are added in a specialized “inner chain” that is independent from main chain</t>
+    <t xml:space="preserve">Orphan rate and all other basic properties of main chain remain unchanged, any significant changes are added in a specialized “inner chain” that is independent from main chain, increased orphan rates are also moved into the inner chain, which is supplementary and creates added value</t>
   </si>
   <si>
     <t xml:space="preserve">(9)</t>
@@ -699,7 +850,7 @@
     <t xml:space="preserve">(11)</t>
   </si>
   <si>
-    <t xml:space="preserve">Since Infrastructure Blocks heavily touch base consensus, it is expected that they will require a lot of changes to base consensus code</t>
+    <t xml:space="preserve">Since Infrastructure Blocks heavily touch base consensus, it is expected that they will require a lot of changes to base consensus code and some tweaking of existing services</t>
   </si>
   <si>
     <t xml:space="preserve">(12)</t>
@@ -717,7 +868,7 @@
     <t xml:space="preserve">(14)</t>
   </si>
   <si>
-    <t xml:space="preserve">How convenient it is to mine on small scale, comparing to default, meaning: how small are interval times between any coin is mined</t>
+    <t xml:space="preserve">How convenient it is to mine on small scale, comparing to default, meaning: how small are interval times between mining any coin</t>
   </si>
   <si>
     <t xml:space="preserve">(15)</t>
@@ -753,19 +904,43 @@
     <t xml:space="preserve">(20)</t>
   </si>
   <si>
-    <t xml:space="preserve">Infrastructure Blocks introduce a new “sub-bitcoin” coin that is mined along normal Bitcoin and used to pay for fast-finality transactions, increasing miner profits; it is logically expected to increase market activity because the new coin has will be traded separately on BCH DEXes and centralized exchanges</t>
+    <t xml:space="preserve">Infrastructure Blocks introduce a new “sub-bitcoin” coin that is mined along normal Bitcoin and used to pay for fast-finality transactions, increasing miner profits; it is logically expected to increase market activity because the new coin will be traded separately on BCH DEXes and centralized exchanges</t>
   </si>
   <si>
     <t xml:space="preserve">(21)</t>
   </si>
   <si>
-    <t xml:space="preserve">It should be on average 5 times easier for any solo miner to mine any kind of block to achieve profit</t>
+    <t xml:space="preserve">It should be on average 5 times easier for any solo miner to mine any kind of block to achieve income</t>
   </si>
   <si>
     <t xml:space="preserve">(22)</t>
   </si>
   <si>
-    <t xml:space="preserve">It should be on average 60 times easier for any solo miner to mine any kind of block to achieve profit</t>
+    <t xml:space="preserve">It should be on average 60 times easier for any solo miner to mine any kind of block to achieve income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The inner chain of Infrastructure Blocks independently mines its own CashToken coin that, after it achieves value, will be used as additional miner profit source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initially, assuming SPV compatibility scheme is implemented well, Infrastructure Blocks implementation can be postponed by simply using normal 10-minute Blocks and 0-conf: this should require no extra work for many use cases. Full implementation can be done later at convenience.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mining can be continued as usual with minimum changes. But gaining extra profit from Inner Chain token payout can take extra work to setup.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tailstorm punishes some miners’ payout and turns whole inner workings of Nakamoto Consensus upside down. It is a completely new technology, not tested in practice. It is therefore impossible to predict how much work, configuration, trial and error it will take for miners to continue to have stable income</t>
   </si>
   <si>
     <t xml:space="preserve">Sources of information used:</t>
@@ -1001,7 +1176,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1024,6 +1199,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1059,6 +1238,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1281,11 +1464,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N1048576"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="30.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="36.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="27.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="27.47"/>
@@ -1317,7 +1500,7 @@
       <c r="B2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3"/>
+      <c r="C2" s="6"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -1328,19 +1511,19 @@
       <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="10" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1348,19 +1531,19 @@
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="11" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="10" t="s">
         <v>14</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -1371,19 +1554,19 @@
       <c r="B5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="10" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1391,19 +1574,19 @@
       <c r="B6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="10" t="s">
+      <c r="D6" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>23</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="10" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1411,19 +1594,19 @@
       <c r="B7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="11" t="s">
         <v>27</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="10" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1431,19 +1614,19 @@
       <c r="B8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>29</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="10" t="s">
         <v>14</v>
       </c>
       <c r="H8" s="2" t="s">
@@ -1454,19 +1637,19 @@
       <c r="B9" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>34</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H9" s="2" t="s">
@@ -1477,19 +1660,19 @@
       <c r="B10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>38</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H10" s="2" t="s">
@@ -1500,747 +1683,1023 @@
       <c r="B11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="D11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="11" t="s">
         <v>14</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="9" t="s">
-        <v>41</v>
+      <c r="G11" s="10" t="s">
+        <v>42</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="C13" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="D13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>23</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>49</v>
+      <c r="C14" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>50</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="C15" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E15" s="14" t="s">
-        <v>52</v>
+      <c r="D15" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>53</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="14"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="14"/>
-      <c r="G16" s="7"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="15"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="G17" s="9"/>
+        <v>56</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="G17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>57</v>
+      <c r="D18" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>58</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D19" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="C19" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>22</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D20" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="C20" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="15" t="s">
         <v>65</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>66</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>22</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="C22" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E22" s="10" t="s">
         <v>22</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="10" t="s">
         <v>22</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G23" s="9"/>
+      <c r="G23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G24" s="9"/>
-    </row>
-    <row r="26" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
-        <v>72</v>
-      </c>
+      <c r="B24" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="27" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
-        <v>74</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="28" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="D28" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="29" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
-        <v>78</v>
-      </c>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
-        <v>79</v>
+        <v>86</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="B30" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="16"/>
-    </row>
-    <row r="31" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
+      <c r="B30" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="14" t="s">
         <v>82</v>
       </c>
+      <c r="F30" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="B32" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="16"/>
+      <c r="B32" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="B33" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="17"/>
-      <c r="M33" s="17"/>
-      <c r="N33" s="17"/>
+      <c r="B33" s="0"/>
+      <c r="C33" s="0"/>
+      <c r="D33" s="0"/>
+      <c r="E33" s="0"/>
+      <c r="F33" s="0"/>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="B34" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="16"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B35" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
+      <c r="G34" s="10"/>
     </row>
     <row r="36" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15" t="s">
-        <v>92</v>
+      <c r="A36" s="17" t="s">
+        <v>94</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="s">
-        <v>94</v>
+      <c r="A37" s="17" t="s">
+        <v>96</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="s">
-        <v>96</v>
+      <c r="A38" s="17" t="s">
+        <v>98</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="s">
-        <v>98</v>
+      <c r="A39" s="17" t="s">
+        <v>100</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="C40" s="16"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="16"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="16"/>
+      <c r="A40" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="18"/>
+      <c r="M40" s="18"/>
+      <c r="N40" s="18"/>
     </row>
     <row r="41" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="15" t="s">
-        <v>102</v>
+      <c r="A41" s="17" t="s">
+        <v>104</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="B42" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="16"/>
-      <c r="G42" s="16"/>
-      <c r="H42" s="16"/>
-      <c r="I42" s="16"/>
-      <c r="J42" s="16"/>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="16"/>
+      <c r="A42" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="18"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="18"/>
+      <c r="J42" s="18"/>
+      <c r="K42" s="18"/>
+      <c r="L42" s="18"/>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="B43" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="C43" s="16"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
-      <c r="F43" s="16"/>
-      <c r="G43" s="16"/>
-      <c r="H43" s="16"/>
-      <c r="I43" s="16"/>
-      <c r="J43" s="16"/>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="16"/>
+      <c r="A43" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C43" s="19"/>
+      <c r="D43" s="19"/>
+      <c r="E43" s="19"/>
+      <c r="F43" s="19"/>
+      <c r="G43" s="19"/>
+      <c r="H43" s="19"/>
+      <c r="I43" s="19"/>
+      <c r="J43" s="19"/>
+      <c r="K43" s="19"/>
+      <c r="L43" s="19"/>
+      <c r="M43" s="19"/>
+      <c r="N43" s="19"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="B44" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="C44" s="16"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
-      <c r="F44" s="16"/>
-      <c r="G44" s="16"/>
-      <c r="H44" s="16"/>
-      <c r="I44" s="16"/>
-      <c r="J44" s="16"/>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="16"/>
+      <c r="A44" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="18"/>
+      <c r="J44" s="18"/>
+      <c r="K44" s="18"/>
+      <c r="L44" s="18"/>
+      <c r="M44" s="18"/>
+      <c r="N44" s="18"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="B45" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="C45" s="16"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="16"/>
-      <c r="G45" s="16"/>
-      <c r="H45" s="16"/>
-      <c r="I45" s="16"/>
-      <c r="J45" s="16"/>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="16"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="s">
+      <c r="A45" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="B46" s="16" t="s">
+      <c r="B45" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="C46" s="16"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
-      <c r="F46" s="16"/>
-      <c r="G46" s="16"/>
-      <c r="H46" s="16"/>
-      <c r="I46" s="16"/>
-      <c r="J46" s="16"/>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="16"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="s">
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="18"/>
+      <c r="J45" s="18"/>
+      <c r="K45" s="18"/>
+      <c r="L45" s="18"/>
+      <c r="M45" s="18"/>
+      <c r="N45" s="18"/>
+    </row>
+    <row r="46" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="B47" s="16" t="s">
+      <c r="B46" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C47" s="16"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
-      <c r="F47" s="16"/>
-      <c r="G47" s="16"/>
-      <c r="H47" s="16"/>
-      <c r="I47" s="16"/>
-      <c r="J47" s="16"/>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="16"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15"/>
-      <c r="B48" s="16"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="18" t="s">
+    </row>
+    <row r="47" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="17" t="s">
         <v>116</v>
       </c>
+      <c r="B47" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="48" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="49" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="17" t="s">
+        <v>120</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="16"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="C51" s="15"/>
-      <c r="D51" s="15"/>
-      <c r="E51" s="15"/>
-      <c r="F51" s="15"/>
-      <c r="G51" s="15"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="20"/>
-      <c r="J51" s="20"/>
-      <c r="K51" s="20"/>
+      <c r="A50" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="18"/>
+      <c r="J50" s="18"/>
+      <c r="K50" s="18"/>
+      <c r="L50" s="18"/>
+      <c r="M50" s="18"/>
+      <c r="N50" s="18"/>
+    </row>
+    <row r="51" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="C52" s="21"/>
-      <c r="D52" s="21"/>
-      <c r="E52" s="21"/>
-      <c r="F52" s="21"/>
-      <c r="G52" s="21"/>
-      <c r="H52" s="21"/>
-      <c r="I52" s="21"/>
-      <c r="J52" s="21"/>
-      <c r="K52" s="21"/>
+      <c r="A52" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="B52" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C52" s="18"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="18"/>
+      <c r="F52" s="18"/>
+      <c r="G52" s="18"/>
+      <c r="H52" s="18"/>
+      <c r="I52" s="18"/>
+      <c r="J52" s="18"/>
+      <c r="K52" s="18"/>
+      <c r="L52" s="18"/>
+      <c r="M52" s="18"/>
+      <c r="N52" s="18"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="21" t="s">
-        <v>119</v>
-      </c>
-      <c r="C53" s="21"/>
-      <c r="D53" s="21"/>
-      <c r="E53" s="21"/>
-      <c r="F53" s="21"/>
-      <c r="G53" s="21"/>
-      <c r="H53" s="21"/>
-      <c r="I53" s="21"/>
-      <c r="J53" s="21"/>
-      <c r="K53" s="20"/>
+      <c r="A53" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="C53" s="18"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="18"/>
+      <c r="F53" s="18"/>
+      <c r="G53" s="18"/>
+      <c r="H53" s="18"/>
+      <c r="I53" s="18"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="18"/>
+      <c r="M53" s="18"/>
+      <c r="N53" s="18"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="20" t="s">
-        <v>120</v>
-      </c>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
-      <c r="E54" s="20"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="20"/>
-      <c r="J54" s="20"/>
-      <c r="K54" s="20"/>
+      <c r="A54" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B54" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18"/>
+      <c r="I54" s="18"/>
+      <c r="J54" s="18"/>
+      <c r="K54" s="18"/>
+      <c r="L54" s="18"/>
+      <c r="M54" s="18"/>
+      <c r="N54" s="18"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="20"/>
-      <c r="C55" s="15"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="15"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="15"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="20"/>
-      <c r="K55" s="20"/>
+      <c r="A55" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="18"/>
+      <c r="I55" s="18"/>
+      <c r="J55" s="18"/>
+      <c r="K55" s="18"/>
+      <c r="L55" s="18"/>
+      <c r="M55" s="18"/>
+      <c r="N55" s="18"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="C56" s="15"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="20"/>
-      <c r="J56" s="20"/>
-      <c r="K56" s="20"/>
+      <c r="A56" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="B56" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+      <c r="I56" s="18"/>
+      <c r="J56" s="18"/>
+      <c r="K56" s="18"/>
+      <c r="L56" s="18"/>
+      <c r="M56" s="18"/>
+      <c r="N56" s="18"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="C57" s="20"/>
-      <c r="D57" s="20"/>
-      <c r="E57" s="20"/>
-      <c r="F57" s="20"/>
-      <c r="G57" s="20"/>
-      <c r="H57" s="20"/>
-      <c r="I57" s="20"/>
-      <c r="J57" s="20"/>
-      <c r="K57" s="20"/>
+      <c r="A57" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B57" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="18"/>
+      <c r="J57" s="18"/>
+      <c r="K57" s="18"/>
+      <c r="L57" s="18"/>
+      <c r="M57" s="18"/>
+      <c r="N57" s="18"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="C58" s="23"/>
-      <c r="D58" s="23"/>
-      <c r="E58" s="23"/>
-      <c r="F58" s="23"/>
-      <c r="G58" s="23"/>
-      <c r="H58" s="23"/>
-      <c r="I58" s="23"/>
-      <c r="J58" s="23"/>
-      <c r="K58" s="23"/>
+      <c r="A58" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B58" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18"/>
+      <c r="I58" s="18"/>
+      <c r="J58" s="18"/>
+      <c r="K58" s="18"/>
+      <c r="L58" s="18"/>
+      <c r="M58" s="18"/>
+      <c r="N58" s="18"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="20"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
-      <c r="H59" s="20"/>
-      <c r="I59" s="20"/>
-      <c r="J59" s="20"/>
-      <c r="K59" s="20"/>
+      <c r="A59" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B59" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+      <c r="I59" s="18"/>
+      <c r="J59" s="18"/>
+      <c r="K59" s="18"/>
+      <c r="L59" s="18"/>
+      <c r="M59" s="18"/>
+      <c r="N59" s="18"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="C60" s="22"/>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
-      <c r="G60" s="22"/>
-      <c r="H60" s="22"/>
-      <c r="I60" s="22"/>
-      <c r="J60" s="22"/>
-      <c r="K60" s="22"/>
+      <c r="A60" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="B60" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+      <c r="I60" s="18"/>
+      <c r="J60" s="18"/>
+      <c r="K60" s="18"/>
+      <c r="L60" s="18"/>
+      <c r="M60" s="18"/>
+      <c r="N60" s="18"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="20" t="s">
-        <v>125</v>
-      </c>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
-      <c r="E61" s="20"/>
-      <c r="F61" s="20"/>
-      <c r="G61" s="20"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="20"/>
-      <c r="K61" s="20"/>
-    </row>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="A61" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="B61" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18"/>
+      <c r="I61" s="18"/>
+      <c r="J61" s="18"/>
+      <c r="K61" s="18"/>
+      <c r="L61" s="18"/>
+      <c r="M61" s="18"/>
+      <c r="N61" s="18"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="17"/>
+      <c r="B62" s="18"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="17"/>
+      <c r="B63" s="18"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="17"/>
+      <c r="B64" s="18"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B65" s="20" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="18"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="C67" s="17"/>
+      <c r="D67" s="17"/>
+      <c r="E67" s="17"/>
+      <c r="F67" s="17"/>
+      <c r="G67" s="17"/>
+      <c r="H67" s="22"/>
+      <c r="I67" s="22"/>
+      <c r="J67" s="22"/>
+      <c r="K67" s="22"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="C68" s="23"/>
+      <c r="D68" s="23"/>
+      <c r="E68" s="23"/>
+      <c r="F68" s="23"/>
+      <c r="G68" s="23"/>
+      <c r="H68" s="23"/>
+      <c r="I68" s="23"/>
+      <c r="J68" s="23"/>
+      <c r="K68" s="23"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B69" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="C69" s="23"/>
+      <c r="D69" s="23"/>
+      <c r="E69" s="23"/>
+      <c r="F69" s="23"/>
+      <c r="G69" s="23"/>
+      <c r="H69" s="23"/>
+      <c r="I69" s="23"/>
+      <c r="J69" s="23"/>
+      <c r="K69" s="22"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B70" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="C70" s="22"/>
+      <c r="D70" s="22"/>
+      <c r="E70" s="22"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="22"/>
+      <c r="H70" s="22"/>
+      <c r="I70" s="22"/>
+      <c r="J70" s="22"/>
+      <c r="K70" s="22"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B71" s="22"/>
+      <c r="C71" s="17"/>
+      <c r="D71" s="17"/>
+      <c r="E71" s="17"/>
+      <c r="F71" s="17"/>
+      <c r="G71" s="17"/>
+      <c r="H71" s="22"/>
+      <c r="I71" s="22"/>
+      <c r="J71" s="22"/>
+      <c r="K71" s="22"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B72" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="C72" s="17"/>
+      <c r="D72" s="17"/>
+      <c r="E72" s="17"/>
+      <c r="F72" s="17"/>
+      <c r="G72" s="17"/>
+      <c r="H72" s="22"/>
+      <c r="I72" s="22"/>
+      <c r="J72" s="22"/>
+      <c r="K72" s="22"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B73" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C73" s="22"/>
+      <c r="D73" s="22"/>
+      <c r="E73" s="22"/>
+      <c r="F73" s="22"/>
+      <c r="G73" s="22"/>
+      <c r="H73" s="22"/>
+      <c r="I73" s="22"/>
+      <c r="J73" s="22"/>
+      <c r="K73" s="22"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="25" t="s">
+        <v>153</v>
+      </c>
+      <c r="C74" s="25"/>
+      <c r="D74" s="25"/>
+      <c r="E74" s="25"/>
+      <c r="F74" s="25"/>
+      <c r="G74" s="25"/>
+      <c r="H74" s="25"/>
+      <c r="I74" s="25"/>
+      <c r="J74" s="25"/>
+      <c r="K74" s="25"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="22"/>
+      <c r="C75" s="17"/>
+      <c r="D75" s="17"/>
+      <c r="E75" s="17"/>
+      <c r="F75" s="17"/>
+      <c r="G75" s="17"/>
+      <c r="H75" s="22"/>
+      <c r="I75" s="22"/>
+      <c r="J75" s="22"/>
+      <c r="K75" s="22"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B76" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="C76" s="24"/>
+      <c r="D76" s="24"/>
+      <c r="E76" s="24"/>
+      <c r="F76" s="24"/>
+      <c r="G76" s="24"/>
+      <c r="H76" s="24"/>
+      <c r="I76" s="24"/>
+      <c r="J76" s="24"/>
+      <c r="K76" s="24"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="C77" s="22"/>
+      <c r="D77" s="22"/>
+      <c r="E77" s="22"/>
+      <c r="F77" s="22"/>
+      <c r="G77" s="22"/>
+      <c r="H77" s="22"/>
+      <c r="I77" s="22"/>
+      <c r="J77" s="22"/>
+      <c r="K77" s="22"/>
+    </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="B26:N26"/>
-    <mergeCell ref="B27:N27"/>
-    <mergeCell ref="B28:N28"/>
-    <mergeCell ref="B29:N29"/>
-    <mergeCell ref="B30:N30"/>
-    <mergeCell ref="B31:N31"/>
-    <mergeCell ref="B32:N32"/>
-    <mergeCell ref="B33:N33"/>
-    <mergeCell ref="B34:N34"/>
-    <mergeCell ref="B35:N35"/>
+  <mergeCells count="33">
     <mergeCell ref="B36:N36"/>
     <mergeCell ref="B37:N37"/>
     <mergeCell ref="B38:N38"/>
@@ -2253,16 +2712,30 @@
     <mergeCell ref="B45:N45"/>
     <mergeCell ref="B46:N46"/>
     <mergeCell ref="B47:N47"/>
-    <mergeCell ref="B52:K52"/>
-    <mergeCell ref="B53:J53"/>
-    <mergeCell ref="B54:J54"/>
-    <mergeCell ref="B57:K57"/>
-    <mergeCell ref="B58:K58"/>
-    <mergeCell ref="B60:K60"/>
-    <mergeCell ref="B61:K61"/>
+    <mergeCell ref="B48:N48"/>
+    <mergeCell ref="B49:N49"/>
+    <mergeCell ref="B50:N50"/>
+    <mergeCell ref="B51:N51"/>
+    <mergeCell ref="B52:N52"/>
+    <mergeCell ref="B53:N53"/>
+    <mergeCell ref="B54:N54"/>
+    <mergeCell ref="B55:N55"/>
+    <mergeCell ref="B56:N56"/>
+    <mergeCell ref="B57:N57"/>
+    <mergeCell ref="B58:N58"/>
+    <mergeCell ref="B59:N59"/>
+    <mergeCell ref="B60:N60"/>
+    <mergeCell ref="B61:N61"/>
+    <mergeCell ref="B68:K68"/>
+    <mergeCell ref="B69:J69"/>
+    <mergeCell ref="B70:J70"/>
+    <mergeCell ref="B73:K73"/>
+    <mergeCell ref="B74:K74"/>
+    <mergeCell ref="B76:K76"/>
+    <mergeCell ref="B77:K77"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B58" r:id="rId1" display="https://gitlab.com/ShadowOfHarbringer/infrastructureblocks/-/raw/master/implementation_consequences_v1.5.pdf?ref_type=heads&amp;inline=false"/>
+    <hyperlink ref="B74" r:id="rId1" display="https://gitlab.com/ShadowOfHarbringer/infrastructureblocks/-/raw/master/implementation_consequences_v1.5.pdf?ref_type=heads&amp;inline=false"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>